<commit_message>
Controle de medição: célula fica verde ao digitar x
Formatação condicional nos pavimentos (I10:AG) pinta de #00B050 quando
o valor é "x", como nas abas TORRE originais; painéis congelados em I10;
remove mesclagem de célula única.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0176EKqwb7amr9sfwoHiH6NW
</commit_message>
<xml_diff>
--- a/Controle_Medicao_Fachada_Ed_Jardim.xlsx
+++ b/Controle_Medicao_Fachada_Ed_Jardim.xlsx
@@ -982,7 +982,20 @@
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
@@ -12932,7 +12945,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="125">
+  <mergeCells count="101">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A7:A9"/>
@@ -12954,102 +12967,78 @@
     <mergeCell ref="C11:C16"/>
     <mergeCell ref="D11:D16"/>
     <mergeCell ref="A11:A16"/>
-    <mergeCell ref="B11"/>
     <mergeCell ref="C17:C22"/>
     <mergeCell ref="D17:D22"/>
     <mergeCell ref="A17:A22"/>
-    <mergeCell ref="B17"/>
     <mergeCell ref="C23:C28"/>
     <mergeCell ref="D23:D28"/>
     <mergeCell ref="A23:A28"/>
-    <mergeCell ref="B23"/>
     <mergeCell ref="C29:C34"/>
     <mergeCell ref="D29:D34"/>
     <mergeCell ref="A29:A34"/>
-    <mergeCell ref="B29"/>
     <mergeCell ref="C35:C40"/>
     <mergeCell ref="D35:D40"/>
     <mergeCell ref="A35:A40"/>
-    <mergeCell ref="B35"/>
     <mergeCell ref="C41:C46"/>
     <mergeCell ref="D41:D46"/>
     <mergeCell ref="A41:A46"/>
-    <mergeCell ref="B41"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="C50:C55"/>
     <mergeCell ref="D50:D55"/>
     <mergeCell ref="A50:A55"/>
-    <mergeCell ref="B50"/>
     <mergeCell ref="C56:C61"/>
     <mergeCell ref="D56:D61"/>
     <mergeCell ref="A56:A61"/>
-    <mergeCell ref="B56"/>
     <mergeCell ref="C62:C67"/>
     <mergeCell ref="D62:D67"/>
     <mergeCell ref="A62:A67"/>
-    <mergeCell ref="B62"/>
     <mergeCell ref="B68:E68"/>
     <mergeCell ref="C71:C76"/>
     <mergeCell ref="D71:D76"/>
     <mergeCell ref="A71:A76"/>
-    <mergeCell ref="B71"/>
     <mergeCell ref="C77:C82"/>
     <mergeCell ref="D77:D82"/>
     <mergeCell ref="A77:A82"/>
-    <mergeCell ref="B77"/>
     <mergeCell ref="C83:C88"/>
     <mergeCell ref="D83:D88"/>
     <mergeCell ref="A83:A88"/>
-    <mergeCell ref="B83"/>
     <mergeCell ref="C89:C94"/>
     <mergeCell ref="D89:D94"/>
     <mergeCell ref="A89:A94"/>
-    <mergeCell ref="B89"/>
     <mergeCell ref="C95:C100"/>
     <mergeCell ref="D95:D100"/>
     <mergeCell ref="A95:A100"/>
-    <mergeCell ref="B95"/>
     <mergeCell ref="C101:C106"/>
     <mergeCell ref="D101:D106"/>
     <mergeCell ref="A101:A106"/>
-    <mergeCell ref="B101"/>
     <mergeCell ref="C107:C112"/>
     <mergeCell ref="D107:D112"/>
     <mergeCell ref="A107:A112"/>
-    <mergeCell ref="B107"/>
     <mergeCell ref="C113:C118"/>
     <mergeCell ref="D113:D118"/>
     <mergeCell ref="A113:A118"/>
-    <mergeCell ref="B113"/>
     <mergeCell ref="C119:C124"/>
     <mergeCell ref="D119:D124"/>
     <mergeCell ref="A119:A124"/>
-    <mergeCell ref="B119"/>
     <mergeCell ref="C125:C130"/>
     <mergeCell ref="D125:D130"/>
     <mergeCell ref="A125:A130"/>
-    <mergeCell ref="B125"/>
     <mergeCell ref="B131:E131"/>
     <mergeCell ref="C134:C139"/>
     <mergeCell ref="D134:D139"/>
     <mergeCell ref="A134:A139"/>
-    <mergeCell ref="B134"/>
     <mergeCell ref="C140:C145"/>
     <mergeCell ref="D140:D145"/>
     <mergeCell ref="A140:A145"/>
-    <mergeCell ref="B140"/>
     <mergeCell ref="C146:C151"/>
     <mergeCell ref="D146:D151"/>
     <mergeCell ref="A146:A151"/>
-    <mergeCell ref="B146"/>
     <mergeCell ref="C152:C157"/>
     <mergeCell ref="D152:D157"/>
     <mergeCell ref="A152:A157"/>
-    <mergeCell ref="B152"/>
     <mergeCell ref="C158:C163"/>
     <mergeCell ref="D158:D163"/>
     <mergeCell ref="A158:A163"/>
-    <mergeCell ref="B158"/>
     <mergeCell ref="B164:E164"/>
     <mergeCell ref="A167:B167"/>
     <mergeCell ref="A168:B168"/>
@@ -13059,6 +13048,11 @@
     <mergeCell ref="A172:B172"/>
     <mergeCell ref="A174:AG174"/>
   </mergeCells>
+  <conditionalFormatting sqref="I10:AG173">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:AU174"/>
   </ignoredErrors>

</xml_diff>